<commit_message>
Update Control Tower dashboard
</commit_message>
<xml_diff>
--- a/docs/NEST_MATCH_OUTREACH_MASTER_2026-08-20.xlsx
+++ b/docs/NEST_MATCH_OUTREACH_MASTER_2026-08-20.xlsx
@@ -20,6 +20,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Categories" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Freelancer Categories" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Research Queue" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Week 1 Provider Outreach" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Company Providers'!$A$1:$T$27</definedName>
@@ -31845,6 +31846,379 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
+    <col width="41" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Monday 31 August to Sunday 6 September 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Segment</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Service providers only</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Channels</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>LinkedIn led, WhatsApp fallback</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>15 live verified provider profiles from 30 approaches</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Category breadth target</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>At least 8 different service categories</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Primary metric</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Live verified profiles, not messages sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Pre-send blocker 1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Walk provider registration end to end</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Pre-send blocker 2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Fix multi-category profile: one primary plus two additional categories</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Pre-send blocker 3</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Fix Damiano LinkedIn headline, featured link and first About lines</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Pre-send blocker 4</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Sort provider list into Tier A/B/C</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Tier A</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Providers Lux Oasis currently pays; WhatsApp first; 70-80% expected conversion</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Tier B</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Providers used before or recommended; WhatsApp or LinkedIn; 40-50% expected conversion</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Tier C</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Known companies not used; LinkedIn only; 15-20% expected conversion</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Open item</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Decide founding-provider free-until date before external messages</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Open item</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Write one-page verification standard before using verified heavily</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Open item</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Use ORL profile only as a test; disclose common ownership or set to draft</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Approval rule</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>No WhatsApp, LinkedIn DM, public post or external send without Damiano approval</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Main block</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Second block</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Mon 31 Aug</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Registration test, category fix, LinkedIn profile, tier list</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>8 Tier A WhatsApp messages</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Tue 1 Sep</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>8 Tier A/B WhatsApp messages</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>LinkedIn post and comment replies</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Wed 2 Sep</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>10 Tier C LinkedIn connection requests</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>DM acceptances and build profiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Thu 3 Sep</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Day 3 follow-ups</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>8 more LinkedIn requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Fri 4 Sep</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>DMs to acceptances</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Build profiles and chase trade licences</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Sat 5 Sep</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Phone calls to Tier A replied-but-not-registered contacts</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Build profiles</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Sun 6 Sep</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Numbers review only</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Draft Week 2 operator post</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>